<commit_message>
db scann 9 particiones actualizado
</commit_message>
<xml_diff>
--- a/results/bitacora/9 particiones.xlsx
+++ b/results/bitacora/9 particiones.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeyian PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mavig\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E88DDA-A6C0-4714-A2D0-21076AC7EC8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82038D5F-B437-4041-93A2-FB08B9478665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="26145" windowHeight="19035" xr2:uid="{5C48DCA9-C44A-42ED-B262-D1DF19BF14BF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5C48DCA9-C44A-42ED-B262-D1DF19BF14BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>Valor de K / grupos</t>
   </si>
@@ -91,21 +91,6 @@
   </si>
   <si>
     <t>dendrogram</t>
-  </si>
-  <si>
-    <t>X_PCA.csv</t>
-  </si>
-  <si>
-    <t>4964,3</t>
-  </si>
-  <si>
-    <t>X.csv</t>
-  </si>
-  <si>
-    <t>4786,2,2</t>
-  </si>
-  <si>
-    <t>4983,3,2,2</t>
   </si>
 </sst>
 </file>
@@ -249,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -271,11 +256,133 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="111">
+  <dxfs count="126">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCC0000"/>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCC0000"/>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCC0000"/>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCC0000"/>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCC0000"/>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1475,14 +1582,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465FAB78-C51A-42E5-8E86-EE082C41AADF}">
   <dimension ref="A2:P25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1511,7 +1618,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
         <v>2</v>
       </c>
@@ -1534,7 +1641,7 @@
         <v>1.5899000000000001</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>3</v>
       </c>
@@ -1561,7 +1668,7 @@
         <v>1.5834999999999999</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>4</v>
       </c>
@@ -1590,7 +1697,7 @@
         <v>1.8445</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="8" t="s">
         <v>5</v>
       </c>
@@ -1622,103 +1729,103 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="7">
-        <v>323</v>
+        <v>2</v>
       </c>
       <c r="C9" s="10">
-        <v>3749</v>
+        <v>33</v>
       </c>
       <c r="D9" s="10">
-        <v>74.98</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="10">
         <v>3</v>
       </c>
       <c r="F9" s="10">
-        <v>10</v>
+        <v>4964</v>
       </c>
       <c r="G9" s="10">
-        <v>3.33</v>
+        <v>1654.67</v>
       </c>
       <c r="I9" s="3">
         <v>1</v>
       </c>
-      <c r="J9" s="10">
-        <v>33878.419300000001</v>
-      </c>
-      <c r="K9" s="10">
-        <v>0.71220000000000006</v>
-      </c>
-      <c r="L9" s="10">
-        <v>0.32840000000000003</v>
+      <c r="J9" s="19">
+        <v>4.4170999999999996</v>
+      </c>
+      <c r="K9" s="18">
+        <v>7.6499999999999999E-2</v>
+      </c>
+      <c r="L9" s="19">
+        <v>0.82379999999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="7">
-        <v>819</v>
+        <v>3</v>
       </c>
       <c r="C10" s="10">
-        <v>2951</v>
+        <v>210</v>
       </c>
       <c r="D10" s="10">
-        <v>59.02</v>
+        <v>4.2</v>
       </c>
       <c r="E10" s="10">
         <v>2</v>
       </c>
       <c r="F10" s="10">
-        <v>10</v>
+        <v>4786</v>
       </c>
       <c r="G10" s="10">
-        <v>5</v>
+        <v>2393</v>
       </c>
       <c r="I10" s="3">
         <v>2</v>
       </c>
-      <c r="J10" s="14">
-        <v>40778.623399999997</v>
-      </c>
-      <c r="K10" s="11">
-        <v>0.70609999999999995</v>
-      </c>
-      <c r="L10" s="14">
-        <v>0.29630000000000001</v>
+      <c r="J10" s="19">
+        <v>3.202</v>
+      </c>
+      <c r="K10" s="19">
+        <v>-3.2099999999999997E-2</v>
+      </c>
+      <c r="L10" s="19">
+        <v>1.2083999999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="7">
-        <v>916</v>
+        <v>4</v>
       </c>
       <c r="C11" s="10">
-        <v>2563</v>
+        <v>10</v>
       </c>
       <c r="D11" s="10">
-        <v>51.26</v>
+        <v>0.2</v>
       </c>
       <c r="E11" s="10">
         <v>2</v>
       </c>
       <c r="F11" s="10">
-        <v>10</v>
+        <v>4983</v>
       </c>
       <c r="G11" s="10">
-        <v>5</v>
+        <v>2491.5</v>
       </c>
       <c r="I11" s="3">
         <v>3</v>
       </c>
-      <c r="J11" s="11">
-        <v>30049.062300000001</v>
-      </c>
-      <c r="K11" s="14">
-        <v>0.66479999999999995</v>
-      </c>
-      <c r="L11" s="11">
-        <v>0.3397</v>
+      <c r="J11" s="19">
+        <v>4.9690000000000003</v>
+      </c>
+      <c r="K11" s="19">
+        <v>-0.1893</v>
+      </c>
+      <c r="L11" s="19">
+        <v>0.76849999999999996</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="8" t="s">
         <v>11</v>
       </c>
@@ -1750,7 +1857,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
         <v>17</v>
       </c>
@@ -1779,7 +1886,7 @@
         <v>1.7555000000000001</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="6">
         <v>1</v>
       </c>
@@ -1808,7 +1915,7 @@
         <v>2.0057</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B17" s="6">
         <v>2</v>
       </c>
@@ -1840,7 +1947,7 @@
         <v>2.7753999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B18" s="6">
         <v>3</v>
       </c>
@@ -1860,713 +1967,530 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="16" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16">
-        <v>158</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="16">
-        <v>0.316</v>
-      </c>
-      <c r="D22" s="16">
-        <v>3</v>
-      </c>
-      <c r="E22" s="16">
-        <v>2</v>
-      </c>
-      <c r="F22" s="16">
-        <v>33</v>
-      </c>
-      <c r="G22" s="16">
-        <v>0.66</v>
-      </c>
-      <c r="H22" s="16">
-        <v>3</v>
-      </c>
-      <c r="I22" s="16">
-        <v>4964</v>
-      </c>
-      <c r="J22" s="16">
-        <v>2483.5</v>
-      </c>
-      <c r="K22" s="16">
-        <v>2480.5</v>
-      </c>
-      <c r="L22" s="16">
-        <v>1654.67</v>
-      </c>
-      <c r="M22" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="N22" s="16">
-        <v>0.82379999999999998</v>
-      </c>
-      <c r="O22" s="16">
-        <v>4.4170999999999996</v>
-      </c>
-      <c r="P22" s="16">
-        <v>7.6499999999999999E-2</v>
-      </c>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="20"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="20"/>
+      <c r="P21" s="20"/>
     </row>
-    <row r="23" spans="1:16" s="17" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
-        <v>196</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="17">
-        <v>4.6981000000000002</v>
-      </c>
-      <c r="D23" s="17">
-        <v>2</v>
-      </c>
-      <c r="E23" s="17">
-        <v>3</v>
-      </c>
-      <c r="F23" s="17">
-        <v>210</v>
-      </c>
-      <c r="G23" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="H23" s="17">
-        <v>2</v>
-      </c>
-      <c r="I23" s="17">
-        <v>4786</v>
-      </c>
-      <c r="J23" s="17">
-        <v>1596.67</v>
-      </c>
-      <c r="K23" s="17">
-        <v>2255.1999999999998</v>
-      </c>
-      <c r="L23" s="17">
-        <v>2393</v>
-      </c>
-      <c r="M23" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="N23" s="17">
-        <v>1.2083999999999999</v>
-      </c>
-      <c r="O23" s="17">
-        <v>3.202</v>
-      </c>
-      <c r="P23" s="17">
-        <v>-3.2099999999999997E-2</v>
-      </c>
+    <row r="22" spans="1:16" s="16" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="20"/>
+      <c r="O22" s="20"/>
+      <c r="P22" s="20"/>
     </row>
-    <row r="24" spans="1:16" s="17" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17">
-        <v>149</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="17">
-        <v>0.4395</v>
-      </c>
-      <c r="D24" s="17">
-        <v>2</v>
-      </c>
-      <c r="E24" s="17">
-        <v>4</v>
-      </c>
-      <c r="F24" s="17">
-        <v>10</v>
-      </c>
-      <c r="G24" s="17">
-        <v>0.2</v>
-      </c>
-      <c r="H24" s="17">
-        <v>2</v>
-      </c>
-      <c r="I24" s="17">
-        <v>4983</v>
-      </c>
-      <c r="J24" s="17">
-        <v>1247.5</v>
-      </c>
-      <c r="K24" s="17">
-        <v>2156.69</v>
-      </c>
-      <c r="L24" s="17">
-        <v>2491.5</v>
-      </c>
-      <c r="M24" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="N24" s="17">
-        <v>0.76849999999999996</v>
-      </c>
-      <c r="O24" s="17">
-        <v>4.9690000000000003</v>
-      </c>
-      <c r="P24" s="17">
-        <v>-0.1893</v>
-      </c>
+    <row r="23" spans="1:16" s="17" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20"/>
+      <c r="P23" s="20"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" s="17" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="20"/>
+      <c r="P24" s="20"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="P25" s="18"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="110" priority="160">
+    <cfRule type="expression" dxfId="125" priority="169">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="109" priority="161">
+    <cfRule type="expression" dxfId="124" priority="170">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="108" priority="162">
+    <cfRule type="expression" dxfId="123" priority="171">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="107" priority="157">
+    <cfRule type="expression" dxfId="122" priority="166">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="106" priority="158">
+    <cfRule type="expression" dxfId="121" priority="167">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="105" priority="159">
+    <cfRule type="expression" dxfId="120" priority="168">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="104" priority="154">
+    <cfRule type="expression" dxfId="119" priority="163">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="103" priority="155">
+    <cfRule type="expression" dxfId="118" priority="164">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="102" priority="156">
+    <cfRule type="expression" dxfId="117" priority="165">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="101" priority="151">
+    <cfRule type="expression" dxfId="116" priority="160">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="100" priority="152">
+    <cfRule type="expression" dxfId="115" priority="161">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="99" priority="153">
+    <cfRule type="expression" dxfId="114" priority="162">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="expression" dxfId="98" priority="148">
+    <cfRule type="expression" dxfId="113" priority="157">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="expression" dxfId="97" priority="149">
+    <cfRule type="expression" dxfId="112" priority="158">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="expression" dxfId="96" priority="150">
+    <cfRule type="expression" dxfId="111" priority="159">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" dxfId="95" priority="142">
+    <cfRule type="expression" dxfId="110" priority="151">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" dxfId="94" priority="143">
+    <cfRule type="expression" dxfId="109" priority="152">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" dxfId="93" priority="144">
+    <cfRule type="expression" dxfId="108" priority="153">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="92" priority="136">
+    <cfRule type="expression" dxfId="107" priority="145">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="91" priority="137">
+    <cfRule type="expression" dxfId="106" priority="146">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="90" priority="138">
+    <cfRule type="expression" dxfId="105" priority="147">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="expression" dxfId="89" priority="133">
+    <cfRule type="expression" dxfId="104" priority="142">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="expression" dxfId="88" priority="134">
+    <cfRule type="expression" dxfId="103" priority="143">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="expression" dxfId="87" priority="135">
+    <cfRule type="expression" dxfId="102" priority="144">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="expression" dxfId="86" priority="130">
+    <cfRule type="expression" dxfId="101" priority="139">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="expression" dxfId="85" priority="131">
+    <cfRule type="expression" dxfId="100" priority="140">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="expression" dxfId="84" priority="132">
+    <cfRule type="expression" dxfId="99" priority="141">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="expression" dxfId="83" priority="100">
+    <cfRule type="expression" dxfId="98" priority="109">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="expression" dxfId="82" priority="101">
+    <cfRule type="expression" dxfId="97" priority="110">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="expression" dxfId="81" priority="102">
+    <cfRule type="expression" dxfId="96" priority="111">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9">
-    <cfRule type="expression" dxfId="80" priority="97">
+    <cfRule type="expression" dxfId="95" priority="106">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9">
-    <cfRule type="expression" dxfId="79" priority="98">
+    <cfRule type="expression" dxfId="94" priority="107">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9">
-    <cfRule type="expression" dxfId="78" priority="99">
+    <cfRule type="expression" dxfId="93" priority="108">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="expression" dxfId="77" priority="94">
+    <cfRule type="expression" dxfId="92" priority="103">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="expression" dxfId="76" priority="95">
+    <cfRule type="expression" dxfId="91" priority="104">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="expression" dxfId="75" priority="96">
+    <cfRule type="expression" dxfId="90" priority="105">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F10">
-    <cfRule type="expression" dxfId="74" priority="91">
+    <cfRule type="expression" dxfId="89" priority="100">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F10">
-    <cfRule type="expression" dxfId="73" priority="92">
+    <cfRule type="expression" dxfId="88" priority="101">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F10">
-    <cfRule type="expression" dxfId="72" priority="93">
+    <cfRule type="expression" dxfId="87" priority="102">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="expression" dxfId="71" priority="88">
+    <cfRule type="expression" dxfId="86" priority="97">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="expression" dxfId="70" priority="89">
+    <cfRule type="expression" dxfId="85" priority="98">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="expression" dxfId="69" priority="90">
+    <cfRule type="expression" dxfId="84" priority="99">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11">
-    <cfRule type="expression" dxfId="68" priority="85">
+    <cfRule type="expression" dxfId="83" priority="94">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11">
-    <cfRule type="expression" dxfId="67" priority="86">
+    <cfRule type="expression" dxfId="82" priority="95">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11">
-    <cfRule type="expression" dxfId="66" priority="87">
+    <cfRule type="expression" dxfId="81" priority="96">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9">
-    <cfRule type="expression" dxfId="65" priority="82">
+    <cfRule type="expression" dxfId="80" priority="91">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9">
-    <cfRule type="expression" dxfId="64" priority="83">
+    <cfRule type="expression" dxfId="79" priority="92">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9">
-    <cfRule type="expression" dxfId="63" priority="84">
+    <cfRule type="expression" dxfId="78" priority="93">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10">
-    <cfRule type="expression" dxfId="62" priority="79">
+    <cfRule type="expression" dxfId="77" priority="88">
       <formula>$F10&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10">
-    <cfRule type="expression" dxfId="61" priority="80">
+    <cfRule type="expression" dxfId="76" priority="89">
       <formula>$E10&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10">
-    <cfRule type="expression" dxfId="60" priority="81">
+    <cfRule type="expression" dxfId="75" priority="90">
       <formula>$L10&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11">
-    <cfRule type="expression" dxfId="59" priority="76">
+    <cfRule type="expression" dxfId="74" priority="85">
       <formula>$F11&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11">
-    <cfRule type="expression" dxfId="58" priority="77">
+    <cfRule type="expression" dxfId="73" priority="86">
       <formula>$E11&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11">
-    <cfRule type="expression" dxfId="57" priority="78">
+    <cfRule type="expression" dxfId="72" priority="87">
       <formula>$L11&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="expression" dxfId="56" priority="73">
+    <cfRule type="expression" dxfId="71" priority="82">
       <formula>$F15&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="expression" dxfId="55" priority="74">
+    <cfRule type="expression" dxfId="70" priority="83">
       <formula>$E15&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="expression" dxfId="54" priority="75">
+    <cfRule type="expression" dxfId="69" priority="84">
       <formula>$L15&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="expression" dxfId="53" priority="70">
+    <cfRule type="expression" dxfId="68" priority="79">
       <formula>$F15&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="expression" dxfId="52" priority="71">
+    <cfRule type="expression" dxfId="67" priority="80">
       <formula>$E15&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="expression" dxfId="51" priority="72">
+    <cfRule type="expression" dxfId="66" priority="81">
       <formula>$L15&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K15">
-    <cfRule type="expression" dxfId="50" priority="67">
+    <cfRule type="expression" dxfId="65" priority="76">
       <formula>$F15&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K15">
-    <cfRule type="expression" dxfId="49" priority="68">
+    <cfRule type="expression" dxfId="64" priority="77">
       <formula>$E15&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K15">
-    <cfRule type="expression" dxfId="48" priority="69">
+    <cfRule type="expression" dxfId="63" priority="78">
       <formula>$L15&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="expression" dxfId="47" priority="46">
+    <cfRule type="expression" dxfId="62" priority="55">
       <formula>$F16&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="expression" dxfId="46" priority="47">
+    <cfRule type="expression" dxfId="61" priority="56">
       <formula>$E16&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="expression" dxfId="45" priority="48">
+    <cfRule type="expression" dxfId="60" priority="57">
       <formula>$L16&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="expression" dxfId="44" priority="43">
+    <cfRule type="expression" dxfId="59" priority="52">
       <formula>$F17&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="expression" dxfId="43" priority="44">
+    <cfRule type="expression" dxfId="58" priority="53">
       <formula>$E17&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="expression" dxfId="42" priority="45">
+    <cfRule type="expression" dxfId="57" priority="54">
       <formula>$L17&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="expression" dxfId="41" priority="40">
+    <cfRule type="expression" dxfId="56" priority="49">
       <formula>$F16&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="expression" dxfId="40" priority="41">
+    <cfRule type="expression" dxfId="55" priority="50">
       <formula>$E16&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="expression" dxfId="39" priority="42">
+    <cfRule type="expression" dxfId="54" priority="51">
       <formula>$L16&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="expression" dxfId="38" priority="37">
+    <cfRule type="expression" dxfId="53" priority="46">
       <formula>$F17&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="expression" dxfId="37" priority="38">
+    <cfRule type="expression" dxfId="52" priority="47">
       <formula>$E17&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="expression" dxfId="36" priority="39">
+    <cfRule type="expression" dxfId="51" priority="48">
       <formula>$L17&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="expression" dxfId="35" priority="34">
+    <cfRule type="expression" dxfId="50" priority="43">
       <formula>$F16&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="expression" dxfId="34" priority="35">
+    <cfRule type="expression" dxfId="49" priority="44">
       <formula>$E16&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="expression" dxfId="33" priority="36">
+    <cfRule type="expression" dxfId="48" priority="45">
       <formula>$L16&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="expression" dxfId="32" priority="31">
+    <cfRule type="expression" dxfId="47" priority="40">
       <formula>$F17&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="expression" dxfId="31" priority="32">
+    <cfRule type="expression" dxfId="46" priority="41">
       <formula>$E17&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="expression" dxfId="30" priority="33">
+    <cfRule type="expression" dxfId="45" priority="42">
       <formula>$L17&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L9">
-    <cfRule type="expression" dxfId="29" priority="28">
+  <conditionalFormatting sqref="L9:L11">
+    <cfRule type="expression" dxfId="8" priority="7">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L9">
-    <cfRule type="expression" dxfId="28" priority="29">
+  <conditionalFormatting sqref="L9:L11">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L9">
-    <cfRule type="expression" dxfId="27" priority="30">
+  <conditionalFormatting sqref="L9:L11">
+    <cfRule type="expression" dxfId="6" priority="9">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
-    <cfRule type="expression" dxfId="26" priority="25">
+  <conditionalFormatting sqref="J9:J11">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
-    <cfRule type="expression" dxfId="25" priority="26">
+  <conditionalFormatting sqref="J9:J11">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
-    <cfRule type="expression" dxfId="24" priority="27">
+  <conditionalFormatting sqref="J9:J11">
+    <cfRule type="expression" dxfId="3" priority="6">
       <formula>$L9&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K9">
-    <cfRule type="expression" dxfId="23" priority="22">
+  <conditionalFormatting sqref="K9:K11">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$F9&gt;4000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K9">
-    <cfRule type="expression" dxfId="22" priority="23">
+  <conditionalFormatting sqref="K9:K11">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$E9&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K9">
-    <cfRule type="expression" dxfId="21" priority="24">
+  <conditionalFormatting sqref="K9:K11">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$L9&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
-    <cfRule type="expression" dxfId="20" priority="19">
-      <formula>$F10&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
-    <cfRule type="expression" dxfId="19" priority="20">
-      <formula>$E10&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
-    <cfRule type="expression" dxfId="18" priority="21">
-      <formula>$L10&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
-    <cfRule type="expression" dxfId="17" priority="16">
-      <formula>$F11&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
-    <cfRule type="expression" dxfId="16" priority="17">
-      <formula>$E11&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
-    <cfRule type="expression" dxfId="15" priority="18">
-      <formula>$L11&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K10">
-    <cfRule type="expression" dxfId="14" priority="13">
-      <formula>$F10&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K10">
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>$E10&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K10">
-    <cfRule type="expression" dxfId="12" priority="15">
-      <formula>$L10&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
-    <cfRule type="expression" dxfId="11" priority="10">
-      <formula>$F11&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
-    <cfRule type="expression" dxfId="10" priority="11">
-      <formula>$E11&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
-    <cfRule type="expression" dxfId="9" priority="12">
-      <formula>$L11&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L10">
-    <cfRule type="expression" dxfId="8" priority="7">
-      <formula>$F10&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L10">
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$E10&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L10">
-    <cfRule type="expression" dxfId="6" priority="9">
-      <formula>$L10&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L11">
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>$F11&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L11">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>$E11&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L11">
-    <cfRule type="expression" dxfId="3" priority="6">
-      <formula>$L11&gt;10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A22:P24">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$F22&gt;4000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A22:P24">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$E22&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A22:P24">
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>$L22&gt;10</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>